<commit_message>
after AI usage writing
</commit_message>
<xml_diff>
--- a/data/robust_authorities.xlsx
+++ b/data/robust_authorities.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>sd</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -469,7 +469,7 @@
         <v>2.120771631447417</v>
       </c>
       <c r="E2" t="n">
-        <v>5.188442121819496</v>
+        <v>0.9139910249218606</v>
       </c>
       <c r="F2" t="n">
         <v>4</v>
@@ -496,7 +496,7 @@
         <v>1.428752681723949</v>
       </c>
       <c r="E3" t="n">
-        <v>4.218034309235076</v>
+        <v>0.8961814920712909</v>
       </c>
       <c r="F3" t="n">
         <v>5</v>
@@ -523,7 +523,7 @@
         <v>1.403221616259885</v>
       </c>
       <c r="E4" t="n">
-        <v>6.90143850187207</v>
+        <v>0.5379422608673102</v>
       </c>
       <c r="F4" t="n">
         <v>8</v>
@@ -550,7 +550,7 @@
         <v>1.270190517929817</v>
       </c>
       <c r="E5" t="n">
-        <v>11.51081526664231</v>
+        <v>0.1911276014238752</v>
       </c>
       <c r="F5" t="n">
         <v>9</v>
@@ -577,7 +577,7 @@
         <v>1.250546875328898</v>
       </c>
       <c r="E6" t="n">
-        <v>4.753085974166446</v>
+        <v>0.6961027115713802</v>
       </c>
       <c r="F6" t="n">
         <v>3</v>
@@ -604,7 +604,7 @@
         <v>0.9997716687889028</v>
       </c>
       <c r="E7" t="n">
-        <v>7.296139194236231</v>
+        <v>0.3625406715860183</v>
       </c>
       <c r="F7" t="n">
         <v>3</v>
@@ -631,7 +631,7 @@
         <v>0.9938469014532358</v>
       </c>
       <c r="E8" t="n">
-        <v>4.995075908497397</v>
+        <v>0.5264127694324408</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
@@ -658,7 +658,7 @@
         <v>0.9580126127687927</v>
       </c>
       <c r="E9" t="n">
-        <v>9.428963155144078</v>
+        <v>0.1759818648460932</v>
       </c>
       <c r="F9" t="n">
         <v>7</v>
@@ -685,7 +685,7 @@
         <v>0.9135104469348734</v>
       </c>
       <c r="E10" t="n">
-        <v>8.594315173091436</v>
+        <v>0.2376770477184895</v>
       </c>
       <c r="F10" t="n">
         <v>7</v>
@@ -712,7 +712,7 @@
         <v>0.8695907452555958</v>
       </c>
       <c r="E11" t="n">
-        <v>6.400008660238948</v>
+        <v>0.3594871470476617</v>
       </c>
       <c r="F11" t="n">
         <v>9</v>
@@ -739,7 +739,7 @@
         <v>0.7917769472117669</v>
       </c>
       <c r="E12" t="n">
-        <v>3.860103072316252</v>
+        <v>0.542691440334841</v>
       </c>
       <c r="F12" t="n">
         <v>7</v>
@@ -766,7 +766,7 @@
         <v>0.6792530412739252</v>
       </c>
       <c r="E13" t="n">
-        <v>6.31951738458779</v>
+        <v>0.2843784604308548</v>
       </c>
       <c r="F13" t="n">
         <v>9</v>
@@ -793,7 +793,7 @@
         <v>0.5510557827138076</v>
       </c>
       <c r="E14" t="n">
-        <v>4.250533958353318</v>
+        <v>0.3430055079831903</v>
       </c>
       <c r="F14" t="n">
         <v>5</v>
@@ -806,24 +806,24 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>78006</v>
+        <v>90001</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PARDES HANNA-KARKUR</t>
+          <t>BE'ER SHEVA</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.4574181021710461</v>
+        <v>-0.5606695670872681</v>
       </c>
       <c r="E15" t="n">
-        <v>-3.948481465543202</v>
+        <v>0.2385864928723909</v>
       </c>
       <c r="F15" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -833,24 +833,24 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>90001</v>
+        <v>700000</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BE'ER SHEVA</t>
+          <t>EMEQ HAMA'AYANOT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.5606695670872681</v>
+        <v>-0.6488590597428505</v>
       </c>
       <c r="E16" t="n">
-        <v>-8.140512606237076</v>
+        <v>0.5250168930193428</v>
       </c>
       <c r="F16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -860,24 +860,24 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>700000</v>
+        <v>12716</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>EMEQ HAMA'AYANOT</t>
+          <t>LEHAVIM</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.6488590597428505</v>
+        <v>-0.6850256952820587</v>
       </c>
       <c r="E17" t="n">
-        <v>-3.269837086837388</v>
+        <v>0.3888621459561066</v>
       </c>
       <c r="F17" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -887,24 +887,24 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>12716</v>
+        <v>100000</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LEHAVIM</t>
+          <t>HAGALIL HAELYON</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.6850256952820587</v>
+        <v>-1.686907991803911</v>
       </c>
       <c r="E18" t="n">
-        <v>-3.051208046495349</v>
+        <v>0.4640919103306923</v>
       </c>
       <c r="F18" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -914,24 +914,24 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>100000</v>
+        <v>9449</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HAGALIL HAELYON</t>
+          <t>BASMAT TAB'UN</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D19" t="n">
-        <v>-1.686907991803911</v>
+        <v>-1.833856544958504</v>
       </c>
       <c r="E19" t="n">
-        <v>-9.616929172026051</v>
+        <v>1.015413537463047</v>
       </c>
       <c r="F19" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -941,24 +941,24 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>9449</v>
+        <v>5413</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BASMAT TAB'UN</t>
+          <t>JISR AZ-ZARQA</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>-1.833856544958504</v>
+        <v>-1.882908873118977</v>
       </c>
       <c r="E20" t="n">
-        <v>-4.038382141088347</v>
+        <v>0.4631304468756603</v>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -968,53 +968,26 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>5413</v>
+        <v>10603</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>JISR AZ-ZARQA</t>
+          <t>LAQYE</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D21" t="n">
-        <v>-1.882908873118977</v>
+        <v>-2.078033125016749</v>
       </c>
       <c r="E21" t="n">
-        <v>-10.75659925465267</v>
+        <v>0.39033417477576</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21" t="inlineStr">
-        <is>
-          <t>under-performer</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>10603</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>LAQYE</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" t="n">
-        <v>-2.078033125016749</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-11.90421855760688</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="inlineStr">
         <is>
           <t>under-performer</t>
         </is>

</xml_diff>